<commit_message>
Add login health check, run every 30 minutes with Slack alerts
- Health check suite (tests/healthcheck): UI login and logout on Chrome,
  and the login API, tagged @healthcheck and safe on prod
- Separate healthcheck Playwright project so regular runs don't repeat it
- Workflow healthcheck.yml: every 30 minutes on demo and on demand,
  Chrome only; uploads the report and notifies Slack only on failure
- Slack message title is now configurable (RUN_NAME)
- Document the cases (HC_LOGIN_001-002) and the workflow
</commit_message>
<xml_diff>
--- a/docs/DemoBlaze_Test_Cases.xlsx
+++ b/docs/DemoBlaze_Test_Cases.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="797" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="416">
   <si>
     <t>Module</t>
   </si>
@@ -451,6 +451,45 @@
   </si>
   <si>
     <t>Alert "Your token has expired, please login again."; user shown as logged out</t>
+  </si>
+  <si>
+    <t>HC_LOGIN_001</t>
+  </si>
+  <si>
+    <t>Health check</t>
+  </si>
+  <si>
+    <t>User can log in and out through the UI (every 30 minutes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open the home page
+2. Log in with valid credentials
+3. Log out</t>
+  </si>
+  <si>
+    <t>Home page loads; "Welcome &lt;username&gt;" shown and tokenp_ cookie set; after logout "Log in" is back</t>
+  </si>
+  <si>
+    <t>tests/healthcheck/login.healthcheck.spec.ts</t>
+  </si>
+  <si>
+    <t>Runs on Chrome every 30 minutes (.github/workflows/healthcheck.yml); Slack alert on failure.</t>
+  </si>
+  <si>
+    <t>HC_LOGIN_002</t>
+  </si>
+  <si>
+    <t>Login API issues a token the API accepts (every 30 minutes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. POST /login with valid credentials
+2. POST /check with the returned token</t>
+  </si>
+  <si>
+    <t>/check returns the account username and the same token</t>
+  </si>
+  <si>
+    <t>Runs with HC_LOGIN_001; Slack alert on failure.</t>
   </si>
   <si>
     <t>TC_CART_001</t>
@@ -1806,10 +1845,10 @@
         <v>9</v>
       </c>
       <c r="B2" s="3">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C2" s="3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D2" s="3">
         <v>5</v>
@@ -1824,7 +1863,7 @@
         <v>2</v>
       </c>
       <c r="H2" s="3">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I2" s="3">
         <v>8</v>
@@ -1936,7 +1975,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -2684,6 +2723,76 @@
       </c>
       <c r="K21" s="3" t="s">
         <v>34</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A22" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="H22" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="I22" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="B23" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="E23" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F23" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="G23" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="H23" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="I23" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="J23" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="K23" s="3" t="s">
+        <v>147</v>
       </c>
     </row>
   </sheetData>
@@ -2747,13 +2856,13 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>136</v>
+        <v>148</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>2</v>
@@ -2762,19 +2871,19 @@
         <v>28</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>140</v>
+        <v>152</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>142</v>
+        <v>154</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>34</v>
@@ -2782,13 +2891,13 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>145</v>
+        <v>157</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>2</v>
@@ -2797,19 +2906,19 @@
         <v>28</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>146</v>
+        <v>158</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>147</v>
+        <v>159</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="K3" s="3" t="s">
         <v>34</v>
@@ -2817,13 +2926,13 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>149</v>
+        <v>161</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>150</v>
+        <v>162</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>2</v>
@@ -2832,19 +2941,19 @@
         <v>28</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>151</v>
+        <v>163</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>152</v>
+        <v>164</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>153</v>
+        <v>165</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="K4" s="3" t="s">
         <v>34</v>
@@ -2852,13 +2961,13 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>154</v>
+        <v>166</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>4</v>
@@ -2867,33 +2976,33 @@
         <v>49</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>157</v>
+        <v>169</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>158</v>
+        <v>170</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>159</v>
+        <v>171</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>160</v>
+        <v>172</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>162</v>
+        <v>174</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>2</v>
@@ -2902,19 +3011,19 @@
         <v>28</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>163</v>
+        <v>175</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>164</v>
+        <v>176</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>165</v>
+        <v>177</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="K6" s="3" t="s">
         <v>34</v>
@@ -2922,13 +3031,13 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>4</v>
@@ -2937,19 +3046,19 @@
         <v>49</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>170</v>
+        <v>182</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>34</v>
@@ -2957,13 +3066,13 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>171</v>
+        <v>183</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>172</v>
+        <v>184</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>173</v>
+        <v>185</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>4</v>
@@ -2972,19 +3081,19 @@
         <v>69</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>174</v>
+        <v>186</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>175</v>
+        <v>187</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>176</v>
+        <v>188</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>34</v>
@@ -2992,13 +3101,13 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>177</v>
+        <v>189</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>179</v>
+        <v>191</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>2</v>
@@ -3007,19 +3116,19 @@
         <v>49</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>168</v>
+        <v>180</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>180</v>
+        <v>192</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>181</v>
+        <v>193</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>34</v>
@@ -3027,13 +3136,13 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>182</v>
+        <v>194</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>183</v>
+        <v>195</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>2</v>
@@ -3042,19 +3151,19 @@
         <v>49</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>184</v>
+        <v>196</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>185</v>
+        <v>197</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>187</v>
+        <v>199</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>34</v>
@@ -3062,13 +3171,13 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>188</v>
+        <v>200</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>189</v>
+        <v>201</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>2</v>
@@ -3077,19 +3186,19 @@
         <v>28</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>190</v>
+        <v>202</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>191</v>
+        <v>203</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>193</v>
+        <v>205</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="K11" s="3" t="s">
         <v>34</v>
@@ -3097,13 +3206,13 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>4</v>
@@ -3112,33 +3221,33 @@
         <v>49</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>196</v>
+        <v>208</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>197</v>
+        <v>209</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>198</v>
+        <v>210</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>199</v>
+        <v>211</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>143</v>
+        <v>155</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>200</v>
+        <v>212</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>201</v>
+        <v>213</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>137</v>
+        <v>149</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>202</v>
+        <v>214</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>4</v>
@@ -3147,16 +3256,16 @@
         <v>69</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>204</v>
+        <v>216</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>8</v>
@@ -3167,13 +3276,13 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>178</v>
+        <v>190</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>206</v>
+        <v>218</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>2</v>
@@ -3182,16 +3291,16 @@
         <v>69</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>207</v>
+        <v>219</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="H14" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>209</v>
+        <v>221</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>8</v>
@@ -3202,13 +3311,13 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>211</v>
+        <v>223</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>4</v>
@@ -3217,16 +3326,16 @@
         <v>69</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>212</v>
+        <v>224</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>214</v>
+        <v>226</v>
       </c>
       <c r="J15" s="3" t="s">
         <v>8</v>
@@ -3237,13 +3346,13 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>215</v>
+        <v>227</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>216</v>
+        <v>228</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>4</v>
@@ -3252,16 +3361,16 @@
         <v>69</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>217</v>
+        <v>229</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>218</v>
+        <v>230</v>
       </c>
       <c r="H16" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>219</v>
+        <v>231</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>8</v>
@@ -3272,13 +3381,13 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>220</v>
+        <v>232</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>222</v>
+        <v>234</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>2</v>
@@ -3287,19 +3396,19 @@
         <v>49</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>224</v>
+        <v>236</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>225</v>
+        <v>237</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="K17" s="3" t="s">
         <v>34</v>
@@ -3307,13 +3416,13 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>227</v>
+        <v>239</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>2</v>
@@ -3322,19 +3431,19 @@
         <v>28</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>223</v>
+        <v>235</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>229</v>
+        <v>241</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>230</v>
+        <v>242</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>231</v>
+        <v>243</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="K18" s="3" t="s">
         <v>34</v>
@@ -3342,13 +3451,13 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>232</v>
+        <v>244</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>233</v>
+        <v>245</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>4</v>
@@ -3357,19 +3466,19 @@
         <v>49</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>235</v>
+        <v>247</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>236</v>
+        <v>248</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>237</v>
+        <v>249</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="K19" s="3" t="s">
         <v>34</v>
@@ -3377,13 +3486,13 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="D20" s="7" t="s">
         <v>3</v>
@@ -3392,19 +3501,19 @@
         <v>28</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>241</v>
+        <v>253</v>
       </c>
       <c r="H20" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>242</v>
+        <v>254</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="K20" s="3" t="s">
         <v>34</v>
@@ -3412,13 +3521,13 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>243</v>
+        <v>255</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>3</v>
@@ -3427,19 +3536,19 @@
         <v>28</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>245</v>
+        <v>257</v>
       </c>
       <c r="H21" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="K21" s="3" t="s">
         <v>34</v>
@@ -3447,13 +3556,13 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>247</v>
+        <v>259</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>248</v>
+        <v>260</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>3</v>
@@ -3462,19 +3571,19 @@
         <v>28</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>249</v>
+        <v>261</v>
       </c>
       <c r="H22" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>246</v>
+        <v>258</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="K22" s="3" t="s">
         <v>34</v>
@@ -3482,13 +3591,13 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>250</v>
+        <v>262</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>251</v>
+        <v>263</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>6</v>
@@ -3497,19 +3606,19 @@
         <v>69</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>252</v>
+        <v>264</v>
       </c>
       <c r="H23" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>253</v>
+        <v>265</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>226</v>
+        <v>238</v>
       </c>
       <c r="K23" s="3" t="s">
         <v>34</v>
@@ -3517,13 +3626,13 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>255</v>
+        <v>267</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>2</v>
@@ -3532,33 +3641,33 @@
         <v>49</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>256</v>
+        <v>268</v>
       </c>
       <c r="H24" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>257</v>
+        <v>269</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>259</v>
+        <v>271</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>261</v>
+        <v>273</v>
       </c>
       <c r="D25" s="7" t="s">
         <v>3</v>
@@ -3567,33 +3676,33 @@
         <v>28</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>262</v>
+        <v>274</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>263</v>
+        <v>275</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>264</v>
+        <v>276</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>258</v>
+        <v>270</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>265</v>
+        <v>277</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>267</v>
+        <v>279</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>3</v>
@@ -3602,33 +3711,33 @@
         <v>28</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>139</v>
+        <v>151</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>268</v>
+        <v>280</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>269</v>
+        <v>281</v>
       </c>
       <c r="I26" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="J26" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="J26" s="3" t="s">
-        <v>258</v>
-      </c>
       <c r="K26" s="3" t="s">
-        <v>271</v>
+        <v>283</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>239</v>
+        <v>251</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>273</v>
+        <v>285</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>3</v>
@@ -3637,33 +3746,33 @@
         <v>49</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>274</v>
+        <v>286</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>275</v>
+        <v>287</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>276</v>
+        <v>288</v>
       </c>
       <c r="J27" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>277</v>
+        <v>289</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>278</v>
+        <v>290</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>279</v>
+        <v>291</v>
       </c>
       <c r="D28" s="9" t="s">
         <v>5</v>
@@ -3672,16 +3781,16 @@
         <v>49</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>280</v>
+        <v>292</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>281</v>
+        <v>293</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>282</v>
+        <v>294</v>
       </c>
       <c r="J28" s="3" t="s">
         <v>8</v>
@@ -3692,13 +3801,13 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>283</v>
+        <v>295</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>221</v>
+        <v>233</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>284</v>
+        <v>296</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>4</v>
@@ -3707,16 +3816,16 @@
         <v>69</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>234</v>
+        <v>246</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>285</v>
+        <v>297</v>
       </c>
       <c r="H29" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>286</v>
+        <v>298</v>
       </c>
       <c r="J29" s="3" t="s">
         <v>8</v>
@@ -3727,13 +3836,13 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>287</v>
+        <v>299</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>288</v>
+        <v>300</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>289</v>
+        <v>301</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>2</v>
@@ -3742,19 +3851,19 @@
         <v>28</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>290</v>
+        <v>302</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>291</v>
+        <v>303</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>292</v>
+        <v>304</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>293</v>
+        <v>305</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>294</v>
+        <v>306</v>
       </c>
       <c r="K30" s="3" t="s">
         <v>34</v>
@@ -3821,13 +3930,13 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>295</v>
+        <v>307</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>297</v>
+        <v>309</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>2</v>
@@ -3839,16 +3948,16 @@
         <v>81</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>298</v>
+        <v>310</v>
       </c>
       <c r="H2" s="3" t="s">
         <v>83</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>299</v>
+        <v>311</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="K2" s="3" t="s">
         <v>34</v>
@@ -3856,13 +3965,13 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>301</v>
+        <v>313</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>302</v>
+        <v>314</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>303</v>
+        <v>315</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>2</v>
@@ -3871,19 +3980,19 @@
         <v>28</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>304</v>
+        <v>316</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>305</v>
+        <v>317</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>306</v>
+        <v>318</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="K3" s="3" t="s">
         <v>34</v>
@@ -3891,13 +4000,13 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>307</v>
+        <v>319</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>308</v>
+        <v>320</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>3</v>
@@ -3909,16 +4018,16 @@
         <v>81</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>309</v>
+        <v>321</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="K4" s="3" t="s">
         <v>34</v>
@@ -3926,13 +4035,13 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>311</v>
+        <v>323</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>312</v>
+        <v>324</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>3</v>
@@ -3944,16 +4053,16 @@
         <v>51</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>313</v>
+        <v>325</v>
       </c>
       <c r="H5" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>314</v>
+        <v>326</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="K5" s="3" t="s">
         <v>34</v>
@@ -3961,13 +4070,13 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>315</v>
+        <v>327</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>296</v>
+        <v>308</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>316</v>
+        <v>328</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>4</v>
@@ -3979,16 +4088,16 @@
         <v>81</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>317</v>
+        <v>329</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>310</v>
+        <v>322</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="K6" s="3" t="s">
         <v>34</v>
@@ -3996,13 +4105,13 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>318</v>
+        <v>330</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>302</v>
+        <v>314</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>319</v>
+        <v>331</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>3</v>
@@ -4014,16 +4123,16 @@
         <v>51</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>320</v>
+        <v>332</v>
       </c>
       <c r="H7" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>321</v>
+        <v>333</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>300</v>
+        <v>312</v>
       </c>
       <c r="K7" s="3" t="s">
         <v>34</v>
@@ -4031,13 +4140,13 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>322</v>
+        <v>334</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>323</v>
+        <v>335</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>324</v>
+        <v>336</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>2</v>
@@ -4049,16 +4158,16 @@
         <v>51</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>325</v>
+        <v>337</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>326</v>
+        <v>338</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>34</v>
@@ -4066,13 +4175,13 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>328</v>
+        <v>340</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>330</v>
+        <v>342</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>2</v>
@@ -4084,16 +4193,16 @@
         <v>51</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>331</v>
+        <v>343</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>332</v>
+        <v>344</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>34</v>
@@ -4101,13 +4210,13 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>333</v>
+        <v>345</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>329</v>
+        <v>341</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>334</v>
+        <v>346</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>3</v>
@@ -4119,16 +4228,16 @@
         <v>51</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>335</v>
+        <v>347</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>336</v>
+        <v>348</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>34</v>
@@ -4136,13 +4245,13 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>337</v>
+        <v>349</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>338</v>
+        <v>350</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>339</v>
+        <v>351</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>2</v>
@@ -4151,19 +4260,19 @@
         <v>28</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>340</v>
+        <v>352</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>341</v>
+        <v>353</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>192</v>
+        <v>204</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>342</v>
+        <v>354</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="K11" s="3" t="s">
         <v>34</v>
@@ -4171,13 +4280,13 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>343</v>
+        <v>355</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>338</v>
+        <v>350</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>344</v>
+        <v>356</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>2</v>
@@ -4186,19 +4295,19 @@
         <v>49</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>345</v>
+        <v>357</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>346</v>
+        <v>358</v>
       </c>
       <c r="H12" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>347</v>
+        <v>359</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="K12" s="3" t="s">
         <v>34</v>
@@ -4206,13 +4315,13 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>348</v>
+        <v>360</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>338</v>
+        <v>350</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>349</v>
+        <v>361</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>5</v>
@@ -4221,19 +4330,19 @@
         <v>28</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>350</v>
+        <v>362</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>351</v>
+        <v>363</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>352</v>
+        <v>364</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="K13" s="3" t="s">
         <v>34</v>
@@ -4241,13 +4350,13 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>353</v>
+        <v>365</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>354</v>
+        <v>366</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>355</v>
+        <v>367</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>2</v>
@@ -4259,16 +4368,16 @@
         <v>81</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>356</v>
+        <v>368</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>186</v>
+        <v>198</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>357</v>
+        <v>369</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="K14" s="3" t="s">
         <v>34</v>
@@ -4276,13 +4385,13 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>358</v>
+        <v>370</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>354</v>
+        <v>366</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>359</v>
+        <v>371</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>3</v>
@@ -4294,16 +4403,16 @@
         <v>51</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>360</v>
+        <v>372</v>
       </c>
       <c r="H15" s="3" t="s">
         <v>51</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>361</v>
+        <v>373</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>327</v>
+        <v>339</v>
       </c>
       <c r="K15" s="3" t="s">
         <v>34</v>
@@ -4338,180 +4447,180 @@
         <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>362</v>
+        <v>374</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>363</v>
+        <v>375</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>364</v>
+        <v>376</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>365</v>
+        <v>377</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>366</v>
+        <v>378</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>367</v>
+        <v>379</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>368</v>
+        <v>380</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>254</v>
+        <v>266</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>370</v>
+        <v>382</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>371</v>
+        <v>383</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>372</v>
+        <v>384</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>373</v>
+        <v>385</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>374</v>
+        <v>386</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>375</v>
+        <v>387</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>266</v>
+        <v>278</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>376</v>
+        <v>388</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>377</v>
+        <v>389</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>378</v>
+        <v>390</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>379</v>
+        <v>391</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>380</v>
+        <v>392</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>375</v>
+        <v>387</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>260</v>
+        <v>272</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>381</v>
+        <v>393</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>382</v>
+        <v>394</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>383</v>
+        <v>395</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>384</v>
+        <v>396</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>385</v>
+        <v>397</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>375</v>
+        <v>387</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>125</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>386</v>
+        <v>398</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>387</v>
+        <v>399</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>388</v>
+        <v>400</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>389</v>
+        <v>401</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>390</v>
+        <v>402</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>369</v>
+        <v>381</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>391</v>
+        <v>403</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>382</v>
+        <v>394</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>383</v>
+        <v>395</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>392</v>
+        <v>404</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>393</v>
+        <v>405</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>394</v>
+        <v>406</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>395</v>
+        <v>407</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>396</v>
+        <v>408</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>397</v>
+        <v>409</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>398</v>
+        <v>410</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>399</v>
+        <v>411</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>400</v>
+        <v>412</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>394</v>
+        <v>406</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>194</v>
+        <v>206</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>401</v>
+        <v>413</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>402</v>
+        <v>414</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>403</v>
+        <v>415</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add KnownBug tags to skip tests with a known defect per environment
A test tagged KnownBug.<env> is skipped on that environment and still runs
on the others; the auto fixture knownBug reports the reason from the test's
issue annotation. Automates TC_ORDER_011 (D-05) and TC_LOGIN_019 (D-04) as
examples.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/DemoBlaze_Test_Cases.xlsx
+++ b/docs/DemoBlaze_Test_Cases.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="416">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="820" uniqueCount="419">
   <si>
     <t>Module</t>
   </si>
@@ -57,6 +57,9 @@
   </si>
   <si>
     <t>"(expected to fail)" = automated check that documents a known defect; it turns red once the defect is fixed.</t>
+  </si>
+  <si>
+    <t>"(known bug: skipped on &lt;env&gt;)" = automated check of a known defect, skipped on that environment until it is fixed.</t>
   </si>
   <si>
     <t>ID</t>
@@ -430,6 +433,9 @@
   </si>
   <si>
     <t>Token is random/opaque and cannot be derived from the username</t>
+  </si>
+  <si>
+    <t>tests/ui/login.spec.ts (known bug: skipped on demo and prod)</t>
   </si>
   <si>
     <t>Observed: token = base64(username + expiry), i.e. forgeable. See Defects D-04.</t>
@@ -950,6 +956,9 @@
   </si>
   <si>
     <t>Order rejected (invalid / expired card)</t>
+  </si>
+  <si>
+    <t>tests/ui/place-order.spec.ts (known bug: skipped on demo)</t>
   </si>
   <si>
     <t>Defect D-05: month/year are not validated.</t>
@@ -1798,7 +1807,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1863,10 +1872,10 @@
         <v>2</v>
       </c>
       <c r="H2" s="3">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I2" s="3">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
@@ -1892,10 +1901,10 @@
         <v>1</v>
       </c>
       <c r="H3" s="3">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="I3" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
@@ -1964,6 +1973,11 @@
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>13</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>14</v>
       </c>
     </row>
   </sheetData>
@@ -1992,807 +2006,807 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D3" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D6" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D9" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D10" s="9" t="s">
         <v>5</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="D13" s="10" t="s">
         <v>6</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="D15" s="10" t="s">
         <v>6</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="J15" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="D17" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="D18" s="9" t="s">
         <v>5</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J18" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D19" s="9" t="s">
         <v>5</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="D20" s="9" t="s">
         <v>5</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>8</v>
+        <v>130</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="D22" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="D23" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
     </row>
   </sheetData>
@@ -2821,1052 +2835,1052 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="D5" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="D8" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="D12" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="J14" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>1</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D15" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="J15" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="D16" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E16" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="G16" s="3" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="H16" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I16" s="3" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K16" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="D17" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I17" s="3" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="J17" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="K17" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D18" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F18" s="3" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="G18" s="3" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="H18" s="3" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="I18" s="3" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="J18" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="K18" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F19" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G19" s="3" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="I19" s="3" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="J19" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="K19" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="D20" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="H20" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I20" s="3" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="J20" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="K20" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D21" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F21" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G21" s="3" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I21" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="J21" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="K21" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="B22" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="D22" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F22" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G22" s="3" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="H22" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I22" s="3" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="J22" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="K22" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" s="3" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="B23" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="D23" s="10" t="s">
         <v>6</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F23" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G23" s="3" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I23" s="3" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="J23" s="3" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="K23" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" s="3" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="B24" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="D24" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F24" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G24" s="3" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="K24" s="3" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="D25" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="K25" s="3" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" s="3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="B26" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="D26" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F26" s="3" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="G26" s="3" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="J26" s="3" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="K26" s="3" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" s="3" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="D27" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="J27" s="3" t="s">
-        <v>8</v>
+        <v>291</v>
       </c>
       <c r="K27" s="3" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" s="3" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>5</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="D28" s="9" t="s">
         <v>5</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F28" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G28" s="3" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="J28" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K28" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" s="3" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="D29" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F29" s="3" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="G29" s="3" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="J29" s="3" t="s">
         <v>8</v>
       </c>
       <c r="K29" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="D30" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="G30" s="3" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="J30" s="3" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="K30" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -3895,527 +3909,527 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="D4" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="D5" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K5" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="D6" s="8" t="s">
         <v>4</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K6" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="D7" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="K7" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="D8" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="K8" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E9" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G9" s="3" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="K9" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="D10" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E10" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G10" s="3" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="K10" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="D11" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E11" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="G11" s="3" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="K11" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="D12" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="G12" s="3" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="H12" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="K12" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="D13" s="9" t="s">
         <v>5</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="G13" s="3" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="H13" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="K13" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="D14" s="6" t="s">
         <v>2</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="H14" s="3" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="I14" s="3" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="J14" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="K14" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="D15" s="7" t="s">
         <v>3</v>
       </c>
       <c r="E15" s="3" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G15" s="3" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="I15" s="3" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="J15" s="3" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="K15" s="3" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -4441,186 +4455,186 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:7" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="E6" s="3" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="E7" s="3" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="G7" s="3" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E8" s="3" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="G8" s="3" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
     </row>
   </sheetData>

</xml_diff>